<commit_message>
Service data model v2 (D-072): seven objects, versioned price book, one job = one payer
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_01JKYsKWsvaEjKCtvVsKEQnj
</commit_message>
<xml_diff>
--- a/docs/Sundial_Estimate_Fields_by_Section.xlsx
+++ b/docs/Sundial_Estimate_Fields_by_Section.xlsx
@@ -2529,10 +2529,14 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Picklist: Price Book / Template / Ad hoc / Field / Migration (default Price Book)</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr"/>
+          <t>Picklist: Price Book / Template / Ad hoc / Field / Migration / Time (default Price Book)</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Time = a billable service call's hours (Added By Service Call points at the call; the labor screen owns the line).</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2572,7 +2576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2806,126 +2810,130 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>Job Type</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Category__c</t>
+          <t>Job_Type__c</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Picklist: Service Call / Inverter / Panel / Battery / EV Charger / Electrical / Roofing / Inspection / Cleaning / Service Plan / Materials / Other</t>
+          <t>Picklist: Solar / Electrical / EV / Commercial</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>GET FROM HARMON: final list, seeded from the HCP export. Unrestricted so the office can add values via the portal admin.</t>
+          <t>List-view filter #1 (2026-09-15): which department's work this item is for. Unrestricted so a tenant can add its own.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Classification</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Service Type</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Description__c</t>
+          <t>Service_Type__c</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Long Text(4000)</t>
+          <t>Picklist: Installation / Repair / Maintenance / Inspection</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Customer-facing text printed on estimates/invoices.</t>
+          <t>List-view filter #2 (2026-09-15): Installation / Repair (+ whatever a tenant adds - unrestricted).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Classification</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Internal Notes</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Internal_Notes__c</t>
+          <t>Category__c</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Long Text(32768)</t>
+          <t>Picklist: Service Call / Inverter / Panel / Battery / EV Charger / Electrical / Roofing / Inspection / Cleaning / Service Plan / Materials / Other</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Never printed. [not cached — detail only]</t>
+          <t>List-view filter #3. GET FROM HARMON: final list, seeded from the HCP export. Unrestricted so the office can add values via the portal admin.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Pricing</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Unit of Measure</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Unit_of_Measure__c</t>
+          <t>Description__c</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Picklist: Each / Hour / Foot / Lot (default Each)</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
+          <t>Long Text(4000)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Customer-facing text printed on estimates/invoices.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Pricing</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Default Quantity</t>
+          <t>Internal Notes</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Default_Quantity__c</t>
+          <t>Internal_Notes__c</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Number(10,2)</t>
+          <t>Long Text(32768)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>e.g. 1.5 hours for the standard service call.</t>
+          <t>Never printed. [not cached — detail only]</t>
         </is>
       </c>
     </row>
@@ -2937,24 +2945,20 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Estimated Hours</t>
+          <t>Unit of Measure</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Estimated_Hours__c</t>
+          <t>Unit_of_Measure__c</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Number(6,2)</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Labor/Product items: default appointment duration when the job is scheduled.</t>
-        </is>
-      </c>
+          <t>Picklist: Each / Hour / Foot / Lot (default Each)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2964,22 +2968,22 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Labor Cost</t>
+          <t>Default Quantity</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Labor_Cost__c</t>
+          <t>Default_Quantity__c</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Currency(16,2)</t>
+          <t>Number(10,2)</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Internal cost (margin reporting).</t>
+          <t>e.g. 1.5 hours for the standard service call.</t>
         </is>
       </c>
     </row>
@@ -2991,22 +2995,22 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Material Cost</t>
+          <t>Estimated Hours</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Material_Cost__c</t>
+          <t>Estimated_Hours__c</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Currency(16,2)</t>
+          <t>Number(6,2)</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Internal cost.</t>
+          <t>Labor/Product items: default appointment duration when the job is scheduled.</t>
         </is>
       </c>
     </row>
@@ -3018,12 +3022,12 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Labor Price</t>
+          <t>Labor Cost</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Labor_Price__c</t>
+          <t>Labor_Cost__c</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -3033,7 +3037,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Sell-side labor portion. Labor items fill only this; Product items fill both.</t>
+          <t>Internal cost (margin reporting).</t>
         </is>
       </c>
     </row>
@@ -3045,12 +3049,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Material Price</t>
+          <t>Material Cost</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Material_Price__c</t>
+          <t>Material_Cost__c</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -3060,34 +3064,34 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Sell-side material portion.</t>
+          <t>Internal cost.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Pricing</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Price__c</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>Formula (Currency)</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>Labor Price + Material Price - the one number the grid shows.</t>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Labor Price</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Labor_Price__c</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Currency(16,2)</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Sell-side labor portion. Labor items fill only this; Product items fill both.</t>
         </is>
       </c>
     </row>
@@ -3099,47 +3103,101 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
+          <t>Material Price</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Material_Price__c</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Currency(16,2)</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Sell-side material portion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Pricing</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Price__c</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Formula (Currency)</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Labor Price + Material Price - the one number the grid shows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Pricing</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
           <t>Taxable</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>Taxable__c</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>Checkbox (default true)</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>Materials default true; labor per tenant tax config. GET FROM HEATHER: how HCP taxed labor vs materials.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>Migration</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>HCP Id</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>HCP_Id__c</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>Text(64) · External ID</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>Housecall Pro price-book id (migration key). [not cached — detail only]</t>
         </is>

</xml_diff>